<commit_message>
Apply student habitation review: AHM-02, AHM-03, SUR-02 not residential; VAP-01 residential
config.HABITATION_REVIEW: new value 'not residential' (verdict ok) for
AHM-02, AHM-03 and SUR-02; VAP-01 set to 'confirmed' (breach). Step 02
re-run: habitation verdicts change only at these four sites (total
breaches 33 -> 34, conditional/check 12 -> 8). Maps and the Google Earth
KML no longer show those sites' buildings as counted dwellings.
v1 charts, workbook, KML and figS5 titles and all v2 figures regenerated.
The config now also finds the KML under its GitHub name (... completer.kml).
03_figures_tables.py gains --no-maps (no imagery download).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016yGYpHzCsTT5hvFUuEY322
</commit_message>
<xml_diff>
--- a/siting_compliance_26Sep/outputs/tables/siting_results.xlsx
+++ b/siting_compliance_26Sep/outputs/tables/siting_results.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrix_2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distances_2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail_2026" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrix_2016" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail_2016" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Habitation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Airports" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protected_areas" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_sources" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matrix_2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Distances_2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Detail_2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Matrix_2016" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Detail_2016" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Habitation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Airports" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Protected_areas" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Rules" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Data_sources" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Parameters" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,17 +576,17 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase</t>
+          <t>Airport / airbase</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -610,17 +610,17 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase</t>
+          <t>Airport / airbase</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -897,22 +897,17 @@
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Pond, Airport / airbase, Flood plain (100-year)</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Habitation</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1006,10 +1001,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
@@ -1019,12 +1014,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>River, Airport / airbase, Flood plain (100-year)</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Habitation</t>
+          <t>River, Habitation, Airport / airbase, Flood plain (100-year)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1623,7 +1613,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'small_airport', 'medium_airport', 'large_airport'}</t>
+          <t>{'large_airport', 'medium_airport', 'small_airport'}</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1673,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/data</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/data</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1745,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/figures</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/figures</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1805,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{'AHM-01': ('confirmed', 'dense housing on the east / south-east edge; industrial units elsewhere (excluded)'), 'AHM-02': ('uncertain', 'Pirana STP to the west (excluded); small structures to the north and south-east may be sheds or huts'), 'AHM-03': ('uncertain', 'many small structures in the walled yard just north; may be a waste-handling / scrap yard, not homes'), 'BHJ-01': ('confirmed', 'houses of the residential area to the south'), 'BHV-01': ('none', 'no buildings inside the 200 m ring'), 'GNR-01': ('confirmed', 'dense cluster of small dwellings along the west edge'), 'JAM-01': ('confirmed', 'residential plots and houses to the south and west'), 'MEH-01': ('confirmed', 'houses to the north-west'), 'RAJ-01': ('none', 'structures in the ring are the processing-plant buildings on the east side'), 'SUR-01': ('confirmed', 'most mapped structures are Bhatar STP units, but dense housing lies inside the ring to the south-west'), 'SUR-02': ('uncertain', 'small cluster south of the southern cell; north side is industrial (excluded)'), 'VAD-01': ('likely', 'scattered houses / farm buildings to the north and west'), 'VAD-02': ('confirmed', 'apartments and houses to the west and south'), 'VAP-01': ('uncertain', 'a few small structures to the south-east; industrial buildings excluded')}</t>
+          <t>{'AHM-01': ('confirmed', 'dense housing on the east / south-east edge; industrial units elsewhere (excluded)'), 'AHM-02': ('not residential', 'student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)'), 'AHM-03': ('not residential', 'student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)'), 'BHJ-01': ('confirmed', 'houses of the residential area to the south'), 'BHV-01': ('none', 'no buildings inside the 200 m ring'), 'GNR-01': ('confirmed', 'dense cluster of small dwellings along the west edge'), 'JAM-01': ('confirmed', 'residential plots and houses to the south and west'), 'MEH-01': ('confirmed', 'houses to the north-west'), 'RAJ-01': ('none', 'structures in the ring are the processing-plant buildings on the east side'), 'SUR-01': ('confirmed', 'most mapped structures are Bhatar STP units, but dense housing lies inside the ring to the south-west'), 'SUR-02': ('not residential', 'student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial'), 'VAD-01': ('likely', 'scattered houses / farm buildings to the north and west'), 'VAD-02': ('confirmed', 'apartments and houses to the west and south'), 'VAP-01': ('confirmed', 'student imagery check 26 Sep: residential buildings within 200 m to the south-east')}</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1841,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>{'motorway_link', 'primary_link', 'motorway', 'primary', 'trunk_link', 'trunk'}</t>
+          <t>{'motorway', 'primary', 'primary_link', 'trunk_link', 'trunk', 'motorway_link'}</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1901,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/home/claude/Locations of landfills in gujurat Completed.kml</t>
+          <t>/home/user/waste-managment-project-1/Locations of landfills in gujurat completer.kml</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1925,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/logs</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/logs</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1949,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>{'RAJ', 'AHM', 'VAD', 'SUR', 'BHV'}</t>
+          <t>{'BHV', 'SUR', 'RAJ', 'VAD', 'AHM'}</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1973,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>{'stream_pool', 'fountain', 'canal', 'ditch', 'stream', 'moat', 'river', 'wastewater', 'drain'}</t>
+          <t>{'drain', 'wastewater', 'river', 'stream_pool', 'moat', 'fountain', 'stream', 'ditch', 'canal'}</t>
         </is>
       </c>
     </row>
@@ -2007,7 +1997,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/outputs</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2057,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>{'', 'lake', 'basin', 'lagoon', 'pond', 'reservoir', 'oxbow'}</t>
+          <t>{'', 'lagoon', 'reservoir', 'oxbow', 'lake', 'basin', 'pond'}</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2069,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/home/claude</t>
+          <t>/home/user/waste-managment-project-1</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2081,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/data/raw</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/data/raw</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2093,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2105,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/scripts</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/scripts</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2117,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/outputs/sites</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs/sites</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2129,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/home/claude/siting_compliance_26Sep/outputs/tables</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs/tables</t>
         </is>
       </c>
     </row>
@@ -2437,9 +2427,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2486,17 +2476,17 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R3" t="n">
         <v>10</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase</t>
+          <t>Airport / airbase</t>
         </is>
       </c>
     </row>
@@ -2526,9 +2516,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2575,17 +2565,17 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R4" t="n">
         <v>10</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase</t>
+          <t>Airport / airbase</t>
         </is>
       </c>
     </row>
@@ -3253,9 +3243,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3302,10 +3292,10 @@
         <v>3</v>
       </c>
       <c r="P12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R12" t="n">
         <v>10</v>
@@ -3315,11 +3305,6 @@
           <t>Pond, Airport / airbase, Flood plain (100-year)</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>Habitation</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3530,9 +3515,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>breach</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3576,10 +3561,10 @@
         </is>
       </c>
       <c r="O15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
         <v>6</v>
@@ -3589,12 +3574,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>River, Airport / airbase, Flood plain (100-year)</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>Habitation</t>
+          <t>River, Habitation, Airport / airbase, Flood plain (100-year)</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3810,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -3893,7 +3873,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -4379,7 +4359,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -4568,7 +4548,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -4629,7 +4609,7 @@
     <col width="58" customWidth="1" min="16" max="16"/>
     <col width="48" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
     <col width="19" customWidth="1" min="21" max="21"/>
     <col width="45" customWidth="1" min="22" max="22"/>
@@ -5750,9 +5730,9 @@
       <c r="K17" t="n">
         <v>48</v>
       </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -5767,12 +5747,12 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Pirana STP to the west (excluded); small structures to the north and south-east may be sheds or huts</t>
+          <t>student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)</t>
         </is>
       </c>
       <c r="U17" t="n">
@@ -6483,9 +6463,9 @@
       <c r="K29" t="n">
         <v>146</v>
       </c>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -6500,12 +6480,12 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>many small structures in the walled yard just north; may be a waste-handling / scrap yard, not homes</t>
+          <t>student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)</t>
         </is>
       </c>
       <c r="U29" t="n">
@@ -12333,9 +12313,9 @@
       <c r="K125" t="n">
         <v>33</v>
       </c>
-      <c r="L125" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
@@ -12350,12 +12330,12 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
         <is>
-          <t>small cluster south of the southern cell; north side is industrial (excluded)</t>
+          <t>student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial</t>
         </is>
       </c>
       <c r="U125" t="n">
@@ -14532,9 +14512,9 @@
       <c r="K161" t="n">
         <v>7</v>
       </c>
-      <c r="L161" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L161" s="3" t="inlineStr">
+        <is>
+          <t>breach</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
@@ -14549,12 +14529,12 @@
       </c>
       <c r="S161" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="T161" t="inlineStr">
         <is>
-          <t>a few small structures to the south-east; industrial buildings excluded</t>
+          <t>student imagery check 26 Sep: residential buildings within 200 m to the south-east</t>
         </is>
       </c>
     </row>
@@ -15052,7 +15032,7 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="60" customWidth="1" min="19" max="19"/>
-    <col width="55" customWidth="1" min="20" max="20"/>
+    <col width="43" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15277,9 +15257,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -15326,17 +15306,17 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3" t="n">
         <v>10</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase, Flood plain (100-year)</t>
+          <t>Airport / airbase, Flood plain (100-year)</t>
         </is>
       </c>
     </row>
@@ -15366,9 +15346,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -15415,17 +15395,17 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R4" t="n">
         <v>10</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase</t>
+          <t>Airport / airbase</t>
         </is>
       </c>
     </row>
@@ -16093,9 +16073,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -16142,10 +16122,10 @@
         <v>2</v>
       </c>
       <c r="P12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R12" t="n">
         <v>10</v>
@@ -16153,11 +16133,6 @@
       <c r="S12" t="inlineStr">
         <is>
           <t>Airport / airbase, Flood plain (100-year)</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>Habitation</t>
         </is>
       </c>
     </row>
@@ -16465,7 +16440,7 @@
     <col width="58" customWidth="1" min="16" max="16"/>
     <col width="48" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
     <col width="19" customWidth="1" min="21" max="21"/>
     <col width="45" customWidth="1" min="22" max="22"/>
@@ -17586,9 +17561,9 @@
       <c r="K17" t="n">
         <v>268</v>
       </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -17603,12 +17578,12 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Pirana STP to the west (excluded); small structures to the north and south-east may be sheds or huts</t>
+          <t>student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)</t>
         </is>
       </c>
       <c r="U17" t="n">
@@ -18319,9 +18294,9 @@
       <c r="K29" t="n">
         <v>74</v>
       </c>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -18336,12 +18311,12 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>many small structures in the walled yard just north; may be a waste-handling / scrap yard, not homes</t>
+          <t>student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)</t>
         </is>
       </c>
       <c r="U29" t="n">
@@ -24159,9 +24134,9 @@
       <c r="K125" t="n">
         <v>36</v>
       </c>
-      <c r="L125" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
@@ -24176,12 +24151,12 @@
       </c>
       <c r="S125" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T125" t="inlineStr">
         <is>
-          <t>small cluster south of the southern cell; north side is industrial (excluded)</t>
+          <t>student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial</t>
         </is>
       </c>
       <c r="U125" t="n">
@@ -26375,12 +26350,12 @@
       </c>
       <c r="S161" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="T161" t="inlineStr">
         <is>
-          <t>a few small structures to the south-east; industrial buildings excluded</t>
+          <t>student imagery check 26 Sep: residential buildings within 200 m to the south-east</t>
         </is>
       </c>
     </row>
@@ -26877,7 +26852,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="28" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
     <col width="25" customWidth="1" min="21" max="21"/>
     <col width="25" customWidth="1" min="22" max="22"/>
@@ -27271,12 +27246,12 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Pirana STP to the west (excluded); small structures to the north and south-east may be sheds or huts</t>
+          <t>student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -27368,12 +27343,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Pirana STP to the west (excluded); small structures to the north and south-east may be sheds or huts</t>
+          <t>student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -27465,12 +27440,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>many small structures in the walled yard just north; may be a waste-handling / scrap yard, not homes</t>
+          <t>student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -27562,12 +27537,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>many small structures in the walled yard just north; may be a waste-handling / scrap yard, not homes</t>
+          <t>student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -29003,12 +28978,12 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>small cluster south of the southern cell; north side is industrial (excluded)</t>
+          <t>student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial</t>
         </is>
       </c>
       <c r="U22" s="3" t="inlineStr">
@@ -29092,12 +29067,12 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>not residential</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>small cluster south of the southern cell; north side is industrial (excluded)</t>
+          <t>student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial</t>
         </is>
       </c>
       <c r="U23" s="3" t="inlineStr">
@@ -29570,12 +29545,12 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>a few small structures to the south-east; industrial buildings excluded</t>
+          <t>student imagery check 26 Sep: residential buildings within 200 m to the south-east</t>
         </is>
       </c>
       <c r="U28" s="3" t="inlineStr">
@@ -29656,12 +29631,12 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>uncertain</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>a few small structures to the south-east; industrial buildings excluded</t>
+          <t>student imagery check 26 Sep: residential buildings within 200 m to the south-east</t>
         </is>
       </c>
       <c r="U29" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Jamnagar: eco-sensitive zone of Khijadiya WLS (5.4 km) counted as a breach
New config.ESZ_REVIEW turns a 1-10 km 'check' into a breach when the site
is confirmed inside the eco-sensitive zone (student, 26 Sep). Step 02
re-run: only JAM-01 R11 changes (2026: 34 -> 35 breaches; 2016: 30 -> 31).
v1 charts, workbook, KML, figS5 titles and all v2 figures regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016yGYpHzCsTT5hvFUuEY322
</commit_message>
<xml_diff>
--- a/siting_compliance_26Sep/outputs/tables/siting_results.xlsx
+++ b/siting_compliance_26Sep/outputs/tables/siting_results.xlsx
@@ -471,7 +471,7 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="37" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -753,25 +753,20 @@
         </is>
       </c>
       <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>3</v>
       </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Highway (NH / SH), Habitation, Airport / airbase</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Critical habitat / eco-fragile area</t>
+          <t>Highway (NH / SH), Habitation, Airport / airbase, Critical habitat / eco-fragile area</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1420,7 +1415,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1574,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1608,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'large_airport', 'medium_airport', 'small_airport'}</t>
+          <t>{'small_airport', 'medium_airport', 'large_airport'}</t>
         </is>
       </c>
     </row>
@@ -1728,442 +1723,454 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FACILITY_BUFFER</t>
+          <t>ESZ_REVIEW</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>{'JAM-01': ('inside ESZ', 'student check 26 Sep: the landfill lies in the eco-sensitive zone of Khijadiya Wildlife Sanctuary (5.4 km)')}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FIG</t>
+          <t>FACILITY_BUFFER</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/figures</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FLOOD_MIN_DEPTH</t>
+          <t>FIG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/figures</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FLOOD_MIN_FRAC</t>
+          <t>FLOOD_MIN_DEPTH</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.0</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GHSL_FUN_URL</t>
+          <t>FLOOD_MIN_FRAC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://jeodpp.jrc.ec.europa.eu/ftp/jrc-opendata/GHSL/GHS_BUILT_C_GLOBE_R2023A/GHS_BUILT_C_FUN_E2018_GLOBE_R2023A_54009_10/V1-0/GHS_BUILT_C_FUN_E2018_GLOBE_R2023A_54009_10_V1_0/GHS_BUILT_C_FUN_E2018_GLOBE_R2023A_54009_10_V1_0.tif</t>
+          <t>0.1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GUJARAT_BBOX</t>
+          <t>GHSL_FUN_URL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>(19.8, 68.0, 24.9, 74.6)</t>
+          <t>https://jeodpp.jrc.ec.europa.eu/ftp/jrc-opendata/GHSL/GHS_BUILT_C_GLOBE_R2023A/GHS_BUILT_C_FUN_E2018_GLOBE_R2023A_54009_10/V1-0/GHS_BUILT_C_FUN_E2018_GLOBE_R2023A_54009_10_V1_0/GHS_BUILT_C_FUN_E2018_GLOBE_R2023A_54009_10_V1_0.tif</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HABITATION_REVIEW</t>
+          <t>GUJARAT_BBOX</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{'AHM-01': ('confirmed', 'dense housing on the east / south-east edge; industrial units elsewhere (excluded)'), 'AHM-02': ('not residential', 'student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)'), 'AHM-03': ('not residential', 'student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)'), 'BHJ-01': ('confirmed', 'houses of the residential area to the south'), 'BHV-01': ('none', 'no buildings inside the 200 m ring'), 'GNR-01': ('confirmed', 'dense cluster of small dwellings along the west edge'), 'JAM-01': ('confirmed', 'residential plots and houses to the south and west'), 'MEH-01': ('confirmed', 'houses to the north-west'), 'RAJ-01': ('none', 'structures in the ring are the processing-plant buildings on the east side'), 'SUR-01': ('confirmed', 'most mapped structures are Bhatar STP units, but dense housing lies inside the ring to the south-west'), 'SUR-02': ('not residential', 'student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial'), 'VAD-01': ('likely', 'scattered houses / farm buildings to the north and west'), 'VAD-02': ('confirmed', 'apartments and houses to the west and south'), 'VAP-01': ('confirmed', 'student imagery check 26 Sep: residential buildings within 200 m to the south-east')}</t>
+          <t>(19.8, 68.0, 24.9, 74.6)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HAB_MIN_BUILDINGS</t>
+          <t>HABITATION_REVIEW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>{'AHM-01': ('confirmed', 'dense housing on the east / south-east edge; industrial units elsewhere (excluded)'), 'AHM-02': ('not residential', 'student imagery check 26 Sep: structures within 200 m are not dwellings (Pirana STP to the west, sheds north and south-east)'), 'AHM-03': ('not residential', 'student imagery check 26 Sep: structures in the walled yard just north are not dwellings (waste-handling / scrap yard)'), 'BHJ-01': ('confirmed', 'houses of the residential area to the south'), 'BHV-01': ('none', 'no buildings inside the 200 m ring'), 'GNR-01': ('confirmed', 'dense cluster of small dwellings along the west edge'), 'JAM-01': ('confirmed', 'residential plots and houses to the south and west'), 'MEH-01': ('confirmed', 'houses to the north-west'), 'RAJ-01': ('none', 'structures in the ring are the processing-plant buildings on the east side'), 'SUR-01': ('confirmed', 'most mapped structures are Bhatar STP units, but dense housing lies inside the ring to the south-west'), 'SUR-02': ('not residential', 'student imagery check 26 Sep: the cluster south of the southern cell is not residential; north side industrial'), 'VAD-01': ('likely', 'scattered houses / farm buildings to the north and west'), 'VAD-02': ('confirmed', 'apartments and houses to the west and south'), 'VAP-01': ('confirmed', 'student imagery check 26 Sep: residential buildings within 200 m to the south-east')}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HAB_SENS</t>
+          <t>HAB_MIN_BUILDINGS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(1, 5, 20)</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HIGHWAY_CLASSES</t>
+          <t>HAB_SENS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>{'motorway', 'primary', 'primary_link', 'trunk_link', 'trunk', 'motorway_link'}</t>
+          <t>(1, 5, 20)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HIGHWAY_REF_REGEX</t>
+          <t>HIGHWAY_CLASSES</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>(?&lt;![A-Za-z])(NH|SH|NE)(?![A-Za-z])</t>
+          <t>{'trunk_link', 'motorway', 'primary', 'trunk', 'motorway_link', 'primary_link'}</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>JRC_FLOOD_CLIPS</t>
+          <t>HIGHWAY_REF_REGEX</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>['ID178_N30_E60_RP100_depth_gujarat.tif', 'ID184_N30_E70_RP100_depth_gujarat.tif']</t>
+          <t>(?&lt;![A-Za-z])(NH|SH|NE)(?![A-Za-z])</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>JRC_PERM_CLIPS</t>
+          <t>JRC_FLOOD_CLIPS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>['ID178_N30_E60_permanent_water_gujarat.tif', 'ID184_N30_E70_permanent_water_gujarat.tif']</t>
+          <t>['ID178_N30_E60_RP100_depth_gujarat.tif', 'ID184_N30_E70_RP100_depth_gujarat.tif']</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>JRC_TILES</t>
+          <t>JRC_PERM_CLIPS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>('ID178_N30_E60', 'ID184_N30_E70')</t>
+          <t>['ID178_N30_E60_permanent_water_gujarat.tif', 'ID184_N30_E70_permanent_water_gujarat.tif']</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KML</t>
+          <t>JRC_TILES</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/Locations of landfills in gujurat completer.kml</t>
+          <t>('ID178_N30_E60', 'ID184_N30_E70')</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LOCAL_RADIUS</t>
+          <t>KML</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2500.0</t>
+          <t>/home/user/waste-managment-project-1/Locations of landfills in gujurat completer.kml</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LOGS</t>
+          <t>LOCAL_RADIUS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/logs</t>
+          <t>2500.0</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MAIN_EPOCH</t>
+          <t>LOGS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/logs</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MAJOR</t>
+          <t>MAIN_EPOCH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>{'BHV', 'SUR', 'RAJ', 'VAD', 'AHM'}</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MIN_POND_M2</t>
+          <t>MAJOR</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>{'BHV', 'SUR', 'AHM', 'VAD', 'RAJ'}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NOT_POND</t>
+          <t>MIN_POND_M2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>{'drain', 'wastewater', 'river', 'stream_pool', 'moat', 'fountain', 'stream', 'ditch', 'canal'}</t>
+          <t>100.0</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OURAIRPORTS_URL</t>
+          <t>NOT_POND</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://davidmegginson.github.io/ourairports-data/airports.csv</t>
+          <t>{'canal', 'fountain', 'stream', 'ditch', 'wastewater', 'drain', 'river', 'moat', 'stream_pool'}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OUT</t>
+          <t>OURAIRPORTS_URL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs</t>
+          <t>https://davidmegginson.github.io/ourairports-data/airports.csv</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OVERPASS_URLS</t>
+          <t>OUT</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>['https://maps.mail.ru/osm/tools/overpass/api/interpreter', 'https://overpass-api.de/api/interpreter', 'https://overpass.kumi.systems/api/interpreter']</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OVERTURE_BUCKET</t>
+          <t>OVERPASS_URLS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>s3://overturemaps-us-west-2/release/{rel}/theme=buildings/type=building/*</t>
+          <t>['https://maps.mail.ru/osm/tools/overpass/api/interpreter', 'https://overpass-api.de/api/interpreter', 'https://overpass.kumi.systems/api/interpreter']</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OVERTURE_RELEASE</t>
+          <t>OVERTURE_BUCKET</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>s3://overturemaps-us-west-2/release/{rel}/theme=buildings/type=building/*</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PARK_LEISURE</t>
+          <t>OVERTURE_RELEASE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>{'park', 'recreation_ground'}</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>POND_WATER_TYPES</t>
+          <t>PARK_LEISURE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>{'', 'lagoon', 'reservoir', 'oxbow', 'lake', 'basin', 'pond'}</t>
+          <t>{'recreation_ground', 'park'}</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PROJECT</t>
+          <t>POND_WATER_TYPES</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1</t>
+          <t>{'', 'pond', 'reservoir', 'oxbow', 'lake', 'lagoon', 'basin'}</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>RAW</t>
+          <t>PROJECT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/data/raw</t>
+          <t>/home/user/waste-managment-project-1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ROOT</t>
+          <t>RAW</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/data/raw</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SCRIPTS</t>
+          <t>ROOT</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/scripts</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SITES_OUT</t>
+          <t>SCRIPTS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs/sites</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/scripts</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TABLES</t>
+          <t>SITES_OUT</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs/tables</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs/sites</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TANK_COMPACTNESS</t>
+          <t>TABLES</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>/home/user/waste-managment-project-1/siting_compliance_26Sep/outputs/tables</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TANK_MIN_M2</t>
+          <t>TANK_COMPACTNESS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.88</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>TANK_MIN_M2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>UTM</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>EPSG:32643</t>
         </is>
@@ -2202,7 +2209,7 @@
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="60" customWidth="1" min="19" max="19"/>
-    <col width="37" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2917,9 +2924,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>breach</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -2928,10 +2935,10 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
         <v>6</v>
@@ -2941,12 +2948,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Highway (NH / SH), Habitation, Airport / airbase</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Critical habitat / eco-fragile area</t>
+          <t>Highway (NH / SH), Habitation, Airport / airbase, Critical habitat / eco-fragile area</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z169"/>
+  <dimension ref="A1:AB169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4616,7 +4618,9 @@
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
     <col width="19" customWidth="1" min="25" max="25"/>
-    <col width="40" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="60" customWidth="1" min="27" max="27"/>
+    <col width="40" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4747,6 +4751,16 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>esz_review</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>esz_note</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>other_protected_land</t>
         </is>
       </c>
@@ -5435,7 +5449,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6185,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6912,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7645,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -8367,10 +8381,10 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
-        </is>
-      </c>
-      <c r="Z60" t="inlineStr">
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
         <is>
           <t>Victoria Nature Park at 5.62 km</t>
         </is>
@@ -9105,7 +9119,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -9825,14 +9839,24 @@
           <t>Khijadiya WLS</t>
         </is>
       </c>
-      <c r="L84" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>breach</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>inside ESZ</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>student check 26 Sep: the landfill lies in the eco-sensitive zone of Khijadiya Wildlife Sanctuary (5.4 km)</t>
         </is>
       </c>
     </row>
@@ -10556,7 +10580,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11304,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -12013,10 +12037,10 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
-        </is>
-      </c>
-      <c r="Z120" t="inlineStr">
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr">
         <is>
           <t>Sarthana Nature Park &amp; Zoo at 11.51 km</t>
         </is>
@@ -12751,7 +12775,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -13484,7 +13508,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -14217,7 +14241,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -14947,7 +14971,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -15747,9 +15771,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>breach</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -15758,10 +15782,10 @@
         </is>
       </c>
       <c r="O8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
         <v>7</v>
@@ -15771,12 +15795,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Habitation, Airport / airbase</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Critical habitat / eco-fragile area</t>
+          <t>Habitation, Airport / airbase, Critical habitat / eco-fragile area</t>
         </is>
       </c>
     </row>
@@ -16419,7 +16438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z169"/>
+  <dimension ref="A1:AB169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16447,7 +16466,9 @@
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
     <col width="19" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="60" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16578,6 +16599,16 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>esz_review</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>esz_note</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>other_protected_land</t>
         </is>
       </c>
@@ -17266,7 +17297,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -18002,7 +18033,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -18729,7 +18760,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -19462,7 +19493,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -20198,7 +20229,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -20931,7 +20962,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -21651,14 +21682,24 @@
           <t>Khijadiya WLS</t>
         </is>
       </c>
-      <c r="L84" s="5" t="inlineStr">
-        <is>
-          <t>check</t>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>breach</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>inside ESZ</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>student check 26 Sep: the landfill lies in the eco-sensitive zone of Khijadiya Wildlife Sanctuary (5.4 km)</t>
         </is>
       </c>
     </row>
@@ -22382,7 +22423,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -23106,7 +23147,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -23839,7 +23880,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -24572,7 +24613,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -25305,7 +25346,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -26038,7 +26079,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>
@@ -26768,7 +26809,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011)</t>
+          <t>OSM protected areas (national parks, sanctuaries, reserves) in Gujarat; inside or &lt; 1 km (minimum ESZ, SC order 3 June 2022) = breach; 1-10 km = check the notified ESZ (10 km default, MoEFCC 2011); confirmed inside the ESZ (config.ESZ_REVIEW) = breach</t>
         </is>
       </c>
     </row>

</xml_diff>